<commit_message>
Document actual Movie Lab UI screenshots
</commit_message>
<xml_diff>
--- a/docs/checklist-self.xlsx
+++ b/docs/checklist-self.xlsx
@@ -4313,7 +4313,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-23 06:19 UTC</t>
+          <t xml:space="preserve">2026-10-23 06:48 UTC</t>
         </is>
       </c>
       <c r="D6" s="3"/>
@@ -4538,12 +4538,12 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">offline-flow.json</t>
+          <t xml:space="preserve">offline-flow.json; 06_top_k3.jpg</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">동일 질문·실제 로컬 검색의 Top-k 1/3: 외부 1/3건(메타데이터 1건 별도). 테스트 벡터 사용</t>
+          <t xml:space="preserve">로컬 모의 검색 Top-k 1/3 외부 1/3건(메타데이터 별도). 실제 앱 설정 5→3→5 확인; 모델 검색 결과 변화는 미실행</t>
         </is>
       </c>
     </row>
@@ -4690,12 +4690,12 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">offline-tests.txt</t>
+          <t xml:space="preserve">offline-tests.txt; 13_missing_key.jpg</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">실제 964편으로 연도·장르·감독 필터 통과. 실제 임베딩 조건탐색 UI 미실행</t>
+          <t xml:space="preserve">로컬 964편 조건 필터 통과. 실제 조건 탐색 제출은 키 없음으로 차단됨; 임베딩 검색 결과 UI 미확인</t>
         </is>
       </c>
     </row>
@@ -4750,12 +4750,12 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui-guidance.json</t>
+          <t xml:space="preserve">ui-guidance.json; 13_empty_index.jpg; 13_missing_key.jpg</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">키 없음·색인 없음 UI 자동 실행 확인. 실제 질문 진행 화면은 미확인</t>
+          <t xml:space="preserve">실제 브라우저의 키 없음·색인 없음 안내 캡처 확인. 실제 질문 진행 화면은 미확인</t>
         </is>
       </c>
     </row>
@@ -4932,12 +4932,12 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">offline-flow.json</t>
+          <t xml:space="preserve">offline-flow.json; 24_sources_license.jpg</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TMDB/Wikipedia 종류 보존 확인. 실제 답변 UI 최종 점검 미실행</t>
+          <t xml:space="preserve">실제 출처 패널에서 TMDB/Wikipedia 구분 확인. 생성 답변의 개별 근거 번호·출처 UI는 미확인</t>
         </is>
       </c>
     </row>
@@ -5084,12 +5084,12 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">../../README.md</t>
+          <t xml:space="preserve">../../README.md; 24_sources_license.jpg</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TMDB/Wikipedia 출처·이용조건·원문/판본 표시 기록</t>
+          <t xml:space="preserve">실제 앱 출처 패널에서 TMDB·위키백과·CC BY-SA 4.0 및 평문 추출·청킹 안내 확인</t>
         </is>
       </c>
     </row>
@@ -5146,12 +5146,12 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">../submission.md</t>
+          <t xml:space="preserve">../screenshots.md; screenshots.json</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">초기 안내 화면 캡처만 가능. 실제 질문·사실검증 등 모든 필수 캡처는 미완료</t>
+          <t xml:space="preserve">실제 캡처 4장(안내 2·출처 1·설정 1) 연결. 질문·진행·사실검증·최종 답변 등 전체 필수 캡처는 미완료</t>
         </is>
       </c>
     </row>

</xml_diff>